<commit_message>
virtuelno okruženje i crtanje mapa
</commit_message>
<xml_diff>
--- a/data/hello_rjesenje.xlsx
+++ b/data/hello_rjesenje.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R63"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -4736,6 +4736,482 @@
       </c>
       <c r="R63" t="n">
         <v>48</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>16DE15</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>VRPB1</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>3977.23</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>371</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>3606.23</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>972.03</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>10</v>
+      </c>
+      <c r="H64" t="n">
+        <v>7</v>
+      </c>
+      <c r="I64" t="n">
+        <v>84</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K64" t="n">
+        <v>39343</v>
+      </c>
+      <c r="L64" t="n">
+        <v>104</v>
+      </c>
+      <c r="M64" t="n">
+        <v>15</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O64" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="P64" t="n">
+        <v>48.98999999999999</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="R64" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>16DE15</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>VRPB1</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>3977.23</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>371</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>3606.23</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>972.03</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>10</v>
+      </c>
+      <c r="H65" t="n">
+        <v>7</v>
+      </c>
+      <c r="I65" t="n">
+        <v>84</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K65" t="n">
+        <v>39343</v>
+      </c>
+      <c r="L65" t="n">
+        <v>104</v>
+      </c>
+      <c r="M65" t="n">
+        <v>15</v>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O65" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="P65" t="n">
+        <v>48.98999999999999</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="R65" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>16DE16</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>VRPB2</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>3788.99</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>4036.0499999999997</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>-247.0599999999999</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>-6.12</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>9</v>
+      </c>
+      <c r="H66" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I66" t="n">
+        <v>77</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K66" t="n">
+        <v>43130</v>
+      </c>
+      <c r="L66" t="n">
+        <v>85</v>
+      </c>
+      <c r="M66" t="n">
+        <v>15</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O66" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="P66" t="n">
+        <v>46.78999999999999</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>67.94</v>
+      </c>
+      <c r="R66" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>16DE17</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>VRPB3</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>3908.9</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>3663.31</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>245.5900000000001</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>9</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="n">
+        <v>74</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K67" t="n">
+        <v>40659</v>
+      </c>
+      <c r="L67" t="n">
+        <v>68</v>
+      </c>
+      <c r="M67" t="n">
+        <v>15</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O67" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="P67" t="n">
+        <v>48.73</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>67.98</v>
+      </c>
+      <c r="R67" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>16DE18</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>VRPB1</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>3977.23</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>371</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>3606.23</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>972.03</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>10</v>
+      </c>
+      <c r="H68" t="n">
+        <v>7</v>
+      </c>
+      <c r="I68" t="n">
+        <v>84</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K68" t="n">
+        <v>39343</v>
+      </c>
+      <c r="L68" t="n">
+        <v>104</v>
+      </c>
+      <c r="M68" t="n">
+        <v>15</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O68" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="P68" t="n">
+        <v>48.98999999999999</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="R68" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>16DE19</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>VRPB2</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>3788.99</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>4036.0499999999997</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>-247.0599999999999</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>-6.12</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>9</v>
+      </c>
+      <c r="H69" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I69" t="n">
+        <v>77</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K69" t="n">
+        <v>43130</v>
+      </c>
+      <c r="L69" t="n">
+        <v>85</v>
+      </c>
+      <c r="M69" t="n">
+        <v>15</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O69" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="P69" t="n">
+        <v>46.78999999999999</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>67.94</v>
+      </c>
+      <c r="R69" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>16DE20</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>VRPB3</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>3908.9</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>3663.31</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>245.5900000000001</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>9</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
+        <v>74</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K70" t="n">
+        <v>40659</v>
+      </c>
+      <c r="L70" t="n">
+        <v>68</v>
+      </c>
+      <c r="M70" t="n">
+        <v>15</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O70" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="P70" t="n">
+        <v>48.73</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>67.98</v>
+      </c>
+      <c r="R70" t="n">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -4749,7 +5225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -5702,6 +6178,414 @@
       </c>
       <c r="R14" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>16DE15</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>VRPB11</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4036.05</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>3977.2299999999996</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>58.82000000000016</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>85</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>24888</v>
+      </c>
+      <c r="L15" t="n">
+        <v>110</v>
+      </c>
+      <c r="M15" t="n">
+        <v>15</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>24.59</v>
+      </c>
+      <c r="P15" t="n">
+        <v>49.34</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>73.95</v>
+      </c>
+      <c r="R15" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>16DE16</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>VRPB22</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3663.31</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>3788.99</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>-125.6799999999998</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>-3.32</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>9</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>68</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>16042</v>
+      </c>
+      <c r="L16" t="n">
+        <v>79</v>
+      </c>
+      <c r="M16" t="n">
+        <v>10</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="P16" t="n">
+        <v>45.20999999999999</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>63.95</v>
+      </c>
+      <c r="R16" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16DE17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>VRPB33</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3362.99</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>3908.9</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>-545.9100000000003</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-13.97</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>7</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>47</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>11518</v>
+      </c>
+      <c r="L17" t="n">
+        <v>48</v>
+      </c>
+      <c r="M17" t="n">
+        <v>10</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="P17" t="n">
+        <v>38.68</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>51.34</v>
+      </c>
+      <c r="R17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>16DE18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>VRPB11</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4036.05</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>3977.2299999999996</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>58.82000000000016</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>10</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>85</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>24888</v>
+      </c>
+      <c r="L18" t="n">
+        <v>110</v>
+      </c>
+      <c r="M18" t="n">
+        <v>15</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>24.59</v>
+      </c>
+      <c r="P18" t="n">
+        <v>49.34</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>73.95</v>
+      </c>
+      <c r="R18" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>16DE19</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>VRPB22</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3663.31</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>3788.99</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>-125.6799999999998</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>-3.32</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>9</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>68</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>16042</v>
+      </c>
+      <c r="L19" t="n">
+        <v>79</v>
+      </c>
+      <c r="M19" t="n">
+        <v>10</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="P19" t="n">
+        <v>45.20999999999999</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>63.95</v>
+      </c>
+      <c r="R19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>16DE20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>VRPB33</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3362.99</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>3908.9</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>-545.9100000000003</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-13.97</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I20" t="n">
+        <v>47</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>11518</v>
+      </c>
+      <c r="L20" t="n">
+        <v>48</v>
+      </c>
+      <c r="M20" t="n">
+        <v>10</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="P20" t="n">
+        <v>38.68</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>51.34</v>
+      </c>
+      <c r="R20" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -5715,7 +6599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -6668,6 +7552,414 @@
       </c>
       <c r="R14" t="n">
         <v>18</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>16DE15</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>VRPBsaUI1</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4116.66</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>3977.2299999999996</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>139.4300000000003</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>3.51</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>84</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>34833</v>
+      </c>
+      <c r="L15" t="n">
+        <v>104</v>
+      </c>
+      <c r="M15" t="n">
+        <v>15</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="P15" t="n">
+        <v>49.95</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>73.88</v>
+      </c>
+      <c r="R15" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>16DE16</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>VRPBsaUI2</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3861.82</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>3788.99</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>72.82999999999993</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1.92</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>9</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>77</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>36332</v>
+      </c>
+      <c r="L16" t="n">
+        <v>85</v>
+      </c>
+      <c r="M16" t="n">
+        <v>15</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="P16" t="n">
+        <v>47.71</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>68.87</v>
+      </c>
+      <c r="R16" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16DE17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>VRPBsaUI3</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3973.7</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>3908.9</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>64.80000000000018</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>10</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>74</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>33002</v>
+      </c>
+      <c r="L17" t="n">
+        <v>68</v>
+      </c>
+      <c r="M17" t="n">
+        <v>15</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="P17" t="n">
+        <v>48.89</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>68.13</v>
+      </c>
+      <c r="R17" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>16DE18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>VRPBsaUI1</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4116.66</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>3977.2299999999996</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>139.4300000000003</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>3.51</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>10</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>84</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>34833</v>
+      </c>
+      <c r="L18" t="n">
+        <v>104</v>
+      </c>
+      <c r="M18" t="n">
+        <v>15</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="P18" t="n">
+        <v>49.95</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>73.88</v>
+      </c>
+      <c r="R18" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>16DE19</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>VRPBsaUI2</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3861.82</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>3788.99</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>72.82999999999993</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1.92</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>9</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>77</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>36332</v>
+      </c>
+      <c r="L19" t="n">
+        <v>85</v>
+      </c>
+      <c r="M19" t="n">
+        <v>15</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="P19" t="n">
+        <v>47.71</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>68.87</v>
+      </c>
+      <c r="R19" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>16DE20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>VRPBsaUI3</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3973.7</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>3908.9</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>64.80000000000018</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="n">
+        <v>74</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>33002</v>
+      </c>
+      <c r="L20" t="n">
+        <v>68</v>
+      </c>
+      <c r="M20" t="n">
+        <v>15</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="P20" t="n">
+        <v>48.89</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>68.13</v>
+      </c>
+      <c r="R20" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -6681,7 +7973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -7636,6 +8928,414 @@
         <v>5</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>16DE15</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>VRPBsaUI11</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4263.77</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>4036.0499999999997</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>227.7199999999998</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>5.64</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>85</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>21317</v>
+      </c>
+      <c r="L15" t="n">
+        <v>110</v>
+      </c>
+      <c r="M15" t="n">
+        <v>15</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="P15" t="n">
+        <v>52.26</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>76.86</v>
+      </c>
+      <c r="R15" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>16DE16</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>VRPBsaUI22</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3663.31</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>3663.31</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>9</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>68</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>15579</v>
+      </c>
+      <c r="L16" t="n">
+        <v>79</v>
+      </c>
+      <c r="M16" t="n">
+        <v>10</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="P16" t="n">
+        <v>45.20999999999999</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>63.95</v>
+      </c>
+      <c r="R16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16DE17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>VRPBsaUI33</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3374.43</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>3362.99</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>11.44000000000005</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.34</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>7</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>47</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>10744</v>
+      </c>
+      <c r="L17" t="n">
+        <v>48</v>
+      </c>
+      <c r="M17" t="n">
+        <v>10</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="P17" t="n">
+        <v>39.16</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>51.83000000000001</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>16DE18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>VRPBsaUI11</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4263.77</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4036.0499999999997</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>227.7199999999998</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>5.64</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>10</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>85</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>21317</v>
+      </c>
+      <c r="L18" t="n">
+        <v>110</v>
+      </c>
+      <c r="M18" t="n">
+        <v>15</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="P18" t="n">
+        <v>52.26</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>76.86</v>
+      </c>
+      <c r="R18" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>16DE19</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>VRPBsaUI22</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3663.31</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>3663.31</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>9</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>68</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>15579</v>
+      </c>
+      <c r="L19" t="n">
+        <v>79</v>
+      </c>
+      <c r="M19" t="n">
+        <v>10</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="P19" t="n">
+        <v>45.20999999999999</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>63.95</v>
+      </c>
+      <c r="R19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>16DE20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>VRPBsaUI33</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3374.43</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>3362.99</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>11.44000000000005</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.34</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>47</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>10744</v>
+      </c>
+      <c r="L20" t="n">
+        <v>48</v>
+      </c>
+      <c r="M20" t="n">
+        <v>10</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="P20" t="n">
+        <v>39.16</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>51.83000000000001</v>
+      </c>
+      <c r="R20" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
promjene za tri razlike izmedju DL i encmark
</commit_message>
<xml_diff>
--- a/data/hello_rjesenje.xlsx
+++ b/data/hello_rjesenje.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:R73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -5212,6 +5212,210 @@
       </c>
       <c r="R70" t="n">
         <v>55</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>16DE21</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>VRPB1</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>3977.23</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>371</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>3606.23</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>972.03</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>10</v>
+      </c>
+      <c r="H71" t="n">
+        <v>7</v>
+      </c>
+      <c r="I71" t="n">
+        <v>84</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K71" t="n">
+        <v>39343</v>
+      </c>
+      <c r="L71" t="n">
+        <v>104</v>
+      </c>
+      <c r="M71" t="n">
+        <v>15</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O71" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="P71" t="n">
+        <v>48.98999999999999</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="R71" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>16DE22</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>VRPB2</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>3788.99</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>4036.0499999999997</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>-247.0599999999999</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>-6.12</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>9</v>
+      </c>
+      <c r="H72" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I72" t="n">
+        <v>77</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K72" t="n">
+        <v>43130</v>
+      </c>
+      <c r="L72" t="n">
+        <v>85</v>
+      </c>
+      <c r="M72" t="n">
+        <v>15</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O72" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="P72" t="n">
+        <v>46.78999999999999</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>67.94</v>
+      </c>
+      <c r="R72" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>16DE23</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>VRPB3</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>3908.9</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>3663.31</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>245.5900000000001</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>9</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" t="n">
+        <v>74</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K73" t="n">
+        <v>40659</v>
+      </c>
+      <c r="L73" t="n">
+        <v>68</v>
+      </c>
+      <c r="M73" t="n">
+        <v>15</v>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O73" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="P73" t="n">
+        <v>48.73</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>67.98</v>
+      </c>
+      <c r="R73" t="n">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -5225,7 +5429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -6586,6 +6790,210 @@
       </c>
       <c r="R20" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>16DE21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>VRPB11</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>4036.05</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>3977.2299999999996</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>58.82000000000016</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>10</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>85</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>24888</v>
+      </c>
+      <c r="L21" t="n">
+        <v>110</v>
+      </c>
+      <c r="M21" t="n">
+        <v>15</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>24.59</v>
+      </c>
+      <c r="P21" t="n">
+        <v>49.34</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>73.95</v>
+      </c>
+      <c r="R21" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>16DE22</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>VRPB22</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3663.31</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3788.99</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>-125.6799999999998</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-3.32</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>9</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>68</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>16042</v>
+      </c>
+      <c r="L22" t="n">
+        <v>79</v>
+      </c>
+      <c r="M22" t="n">
+        <v>10</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="P22" t="n">
+        <v>45.20999999999999</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>63.95</v>
+      </c>
+      <c r="R22" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>16DE23</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>VRPB33</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3362.99</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>3908.9</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>-545.9100000000003</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>-13.97</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>7</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I23" t="n">
+        <v>47</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>11518</v>
+      </c>
+      <c r="L23" t="n">
+        <v>48</v>
+      </c>
+      <c r="M23" t="n">
+        <v>10</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="P23" t="n">
+        <v>38.68</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>51.34</v>
+      </c>
+      <c r="R23" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -6599,7 +7007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -7960,6 +8368,210 @@
       </c>
       <c r="R20" t="n">
         <v>20</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>16DE21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>VRPBsaUI1</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>4116.66</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>3977.2299999999996</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>139.4300000000003</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>3.51</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>10</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>84</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>34833</v>
+      </c>
+      <c r="L21" t="n">
+        <v>104</v>
+      </c>
+      <c r="M21" t="n">
+        <v>15</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="P21" t="n">
+        <v>49.95</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>73.88</v>
+      </c>
+      <c r="R21" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>16DE22</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>VRPBsaUI2</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3861.82</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3788.99</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>72.82999999999993</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1.92</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>9</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>77</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>36332</v>
+      </c>
+      <c r="L22" t="n">
+        <v>85</v>
+      </c>
+      <c r="M22" t="n">
+        <v>15</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="P22" t="n">
+        <v>47.71</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>68.87</v>
+      </c>
+      <c r="R22" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>16DE23</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>VRPBsaUI3</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3973.7</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>3908.9</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>64.80000000000018</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="n">
+        <v>74</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>33002</v>
+      </c>
+      <c r="L23" t="n">
+        <v>68</v>
+      </c>
+      <c r="M23" t="n">
+        <v>15</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="P23" t="n">
+        <v>48.89</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>68.13</v>
+      </c>
+      <c r="R23" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -7973,7 +8585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -9336,6 +9948,210 @@
         <v>5</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>16DE21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>VRPBsaUI11</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>4263.77</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>4036.0499999999997</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>227.7199999999998</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>5.64</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>10</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>85</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>21317</v>
+      </c>
+      <c r="L21" t="n">
+        <v>110</v>
+      </c>
+      <c r="M21" t="n">
+        <v>15</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="P21" t="n">
+        <v>52.26</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>76.86</v>
+      </c>
+      <c r="R21" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>16DE22</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>VRPBsaUI22</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3663.31</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3663.31</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>9</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>68</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>15579</v>
+      </c>
+      <c r="L22" t="n">
+        <v>79</v>
+      </c>
+      <c r="M22" t="n">
+        <v>10</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="P22" t="n">
+        <v>45.20999999999999</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>63.95</v>
+      </c>
+      <c r="R22" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>16DE23</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>VRPBsaUI33</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3374.43</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>3362.99</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>11.44000000000005</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0.34</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>7</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>47</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>10744</v>
+      </c>
+      <c r="L23" t="n">
+        <v>48</v>
+      </c>
+      <c r="M23" t="n">
+        <v>10</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="P23" t="n">
+        <v>39.16</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>51.83000000000001</v>
+      </c>
+      <c r="R23" t="n">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>